<commit_message>
Remove sample answers from candidate scoring
</commit_message>
<xml_diff>
--- a/artifacts/关键标准答案.xlsx
+++ b/artifacts/关键标准答案.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="R5c93d9e3d0674e61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="Rc324b137d3ae4cd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="R0ee7955c30aa41d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="Ra6a69e2b8da74d18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="R074c5a5968504540"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="Ra49390e7ba8441b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="Re7d5e8bd20444320"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="R7e05ae501be748d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="Rc0bc3d2cdade4e57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="Rfa44f156ef9949a8"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>